<commit_message>
Auto update Pengadaan 2026-10-21 08:09:09
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-21).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-21).xlsx
@@ -1531,22 +1531,22 @@
         <v>2561031608</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1228508400</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>1115612710.6</v>
+        <v>1207378630.6</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>1424790940</v>
+        <v>1332523208</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -1905,22 +1905,22 @@
         <v>956612973</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>739420556</v>
+        <v>746310556</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>641617111</v>
+        <v>648466561</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>217192417</v>
+        <v>210302417</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -3369,22 +3369,22 @@
         <v>34441818695</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>417</v>
+        <v>428</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6759755118</v>
+        <v>6858912850</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>417</v>
+        <v>428</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6349451092.6</v>
+        <v>6448066462.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3587</v>
+        <v>3576</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27682063577</v>
+        <v>27582905845</v>
       </c>
     </row>
   </sheetData>
@@ -5370,10 +5370,10 @@
         <v>23566943625.01</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>9496741760.02</v>
+        <v>10766863760.02</v>
       </c>
       <c r="K40" s="10" t="inlineStr">
         <is>
@@ -7546,10 +7546,10 @@
         <v>64085764887.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37704480683.02</v>
+        <v>38974602683.02</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>19</v>
@@ -8378,13 +8378,13 @@
         <v>23</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26394591741</v>
+        <v>26642121741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26394591741</v>
+        <v>26642121741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -12044,13 +12044,13 @@
         <v>161</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>70786680805.01001</v>
+        <v>71034210805.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>66338247005</v>
+        <v>66585777005</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>33</v>

</xml_diff>